<commit_message>
buffer tube stocks tweak
</commit_message>
<xml_diff>
--- a/changes/m4-stocks.xlsx
+++ b/changes/m4-stocks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{072C52C9-4EF0-4558-AA6F-F9065736DF3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A3DE6C5-21DA-4DFC-95CC-4F697D60561C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="129">
+  <si>
+    <t>CURRENT</t>
+  </si>
   <si>
     <t>name</t>
   </si>
@@ -53,9 +56,42 @@
     <t>vertical_recoil</t>
   </si>
   <si>
+    <t>magazine_capacity</t>
+  </si>
+  <si>
+    <t>barrel_deviation</t>
+  </si>
+  <si>
+    <t>bullet_damage</t>
+  </si>
+  <si>
+    <t>bullet_velocity</t>
+  </si>
+  <si>
+    <t>buck_barrel_deviation</t>
+  </si>
+  <si>
+    <t>fire_rate</t>
+  </si>
+  <si>
     <t>price</t>
   </si>
   <si>
+    <t>strength score</t>
+  </si>
+  <si>
+    <t>irl weight</t>
+  </si>
+  <si>
+    <t>weight formula</t>
+  </si>
+  <si>
+    <t>irl price</t>
+  </si>
+  <si>
+    <t>price formula</t>
+  </si>
+  <si>
     <t>hera_arms_cqr_gen2_stock</t>
   </si>
   <si>
@@ -68,349 +104,322 @@
     <t>Hera Arms CQR Gen2 Buttpad</t>
   </si>
   <si>
-    <t>colt_m4a1_receiver_endplate</t>
-  </si>
-  <si>
-    <t>Colt M4A1 Receiver Endplate</t>
+    <t>troy_m7a1_pdw_base_stock</t>
+  </si>
+  <si>
+    <t>Troy M7A1 PDW Base</t>
+  </si>
+  <si>
+    <t>troy_m7a1_pdw_extendable_stock</t>
+  </si>
+  <si>
+    <t>Troy M7A1 PDW Extendable Stock</t>
+  </si>
+  <si>
+    <t>UTG A2 Fixed</t>
+  </si>
+  <si>
+    <t>MDT LSS Fixed</t>
+  </si>
+  <si>
+    <t>MDT Skeleton V5</t>
+  </si>
+  <si>
+    <t>MDT Skeleton V5 Short</t>
+  </si>
+  <si>
+    <t>MDT V5</t>
+  </si>
+  <si>
+    <t>Magpul UBR Gen2 Receiver Extension</t>
+  </si>
+  <si>
+    <t>ubr_gen2_stock</t>
+  </si>
+  <si>
+    <t>Magpul UBR Gen2</t>
+  </si>
+  <si>
+    <t>Magpul PRS Gen2</t>
+  </si>
+  <si>
+    <t>hera_hrs_light_stock</t>
+  </si>
+  <si>
+    <t>Hera HRS Light Fixed</t>
+  </si>
+  <si>
+    <t>sb_tactical_vector_brace</t>
+  </si>
+  <si>
+    <t>SB Tactical Vector Brace</t>
+  </si>
+  <si>
+    <t>si_ar_are_t7_buffer_tube</t>
+  </si>
+  <si>
+    <t>Strike Industries Advanced Receiver Extension T7</t>
+  </si>
+  <si>
+    <t>Fortis LA</t>
+  </si>
+  <si>
+    <t>si_viper_mod1_stock</t>
+  </si>
+  <si>
+    <t>Strike Industries Viper MOD1 Stock</t>
+  </si>
+  <si>
+    <t>viper_rubber_pad</t>
+  </si>
+  <si>
+    <t>Viper Rubber Buttpad</t>
+  </si>
+  <si>
+    <t>Magpul MOE Carbine</t>
+  </si>
+  <si>
+    <t>Magpul MOE Carbine Buttpad</t>
+  </si>
+  <si>
+    <t>ar_tr2_stock</t>
+  </si>
+  <si>
+    <t>AR TR2</t>
+  </si>
+  <si>
+    <t>ar_tr2_pad</t>
+  </si>
+  <si>
+    <t>AR TR2 Buttpad</t>
+  </si>
+  <si>
+    <t>VLTOR EMOD</t>
+  </si>
+  <si>
+    <t>emod_pad</t>
+  </si>
+  <si>
+    <t>EMOD Buttpad</t>
+  </si>
+  <si>
+    <t>Magpul PRS Gen3 Stock</t>
+  </si>
+  <si>
+    <t>prs_adjustable_piece</t>
+  </si>
+  <si>
+    <t>Magpul PRS Gen3 Adjustment Piece</t>
+  </si>
+  <si>
+    <t>prs_gen3_buttpad</t>
+  </si>
+  <si>
+    <t>Magpul PRS Gen3 Buttpad</t>
+  </si>
+  <si>
+    <t>hera_arms_ccs_stock</t>
+  </si>
+  <si>
+    <t>Hera Arms CCS</t>
+  </si>
+  <si>
+    <t>ak12_gen1_std_stock</t>
+  </si>
+  <si>
+    <t>Kalashnikov Concern AK-12 Gen 1</t>
+  </si>
+  <si>
+    <t>lmt_pad</t>
+  </si>
+  <si>
+    <t>LMT Sopmod Buttpad</t>
+  </si>
+  <si>
+    <t>lmt_sopmod</t>
+  </si>
+  <si>
+    <t>LMT Sopmod</t>
+  </si>
+  <si>
+    <t>Brownells XM177 CAR</t>
+  </si>
+  <si>
+    <t>cf_rubber_buttpad</t>
+  </si>
+  <si>
+    <t>CF Rubber Buttpad</t>
+  </si>
+  <si>
+    <t>Magpul STR Carbine</t>
+  </si>
+  <si>
+    <t>Magpul STR Carbine Buttpad</t>
+  </si>
+  <si>
+    <t>Magpul MOE SL-K Carbine</t>
+  </si>
+  <si>
+    <t>Magpul MOE SL-K Carbine Buttpad</t>
+  </si>
+  <si>
+    <t>Daniel Defense Collapsible Milspec Stock</t>
+  </si>
+  <si>
+    <t>Daniel Defense Concave Buttpad</t>
+  </si>
+  <si>
+    <t>CURRENT (SUMMED)</t>
+  </si>
+  <si>
+    <t>Hera Arms CQR Gen2</t>
+  </si>
+  <si>
+    <t>Colt 607 CAR-15 Stock</t>
   </si>
   <si>
     <t>Troy M7A1</t>
   </si>
   <si>
-    <t>leapers_utg_model_15_fixed_a2_ar15_stock</t>
-  </si>
-  <si>
     <t>UTG A2 fixed stock</t>
   </si>
   <si>
-    <t>mdt_lss_stock_adapter</t>
-  </si>
-  <si>
-    <t>MDT LSS Fixed</t>
-  </si>
-  <si>
-    <t>mdt_v5_skeleton_rifle_stock</t>
-  </si>
-  <si>
-    <t>MDT Skeleton V5</t>
-  </si>
-  <si>
-    <t>mdt_v5_skeleton_rifle_stock_short</t>
-  </si>
-  <si>
-    <t>MDT Skeleton V5 Short</t>
-  </si>
-  <si>
-    <t>magpul_ubr_gen2_buffer</t>
-  </si>
-  <si>
     <t>Magpul UBR GEN2</t>
   </si>
   <si>
-    <t>ubr_gen2_stock</t>
-  </si>
-  <si>
-    <t>colt_a2_buffer</t>
-  </si>
-  <si>
-    <t>Colt A2</t>
-  </si>
-  <si>
-    <t>magpul_prs_gen2_stock</t>
-  </si>
-  <si>
-    <t>Magpul PRS Gen2</t>
-  </si>
-  <si>
-    <t>hera_hrs_light_stock</t>
-  </si>
-  <si>
-    <t>Hera HRS Light Fixed</t>
-  </si>
-  <si>
-    <t>colt_m4a1_castlenut</t>
-  </si>
-  <si>
-    <t>Colt M4A1 Castle Nut</t>
-  </si>
-  <si>
-    <t>doublestar_ace_m4_socom_gen4_stock</t>
-  </si>
-  <si>
     <t>Doublestar ACE M4 SOCOM Gen4</t>
   </si>
   <si>
-    <t>doublestar_ace_0.5_recoil_pad</t>
-  </si>
-  <si>
-    <t>sb_tactical_vector_brace</t>
-  </si>
-  <si>
-    <t>SB Tactical Vector Brace</t>
-  </si>
-  <si>
-    <t>si_ar_are_t7_buffer_tube</t>
-  </si>
-  <si>
-    <t>Strike Industries Advanced Receiver Extension T7</t>
-  </si>
-  <si>
-    <t>colt_buffer_tube</t>
-  </si>
-  <si>
-    <t>Colt</t>
-  </si>
-  <si>
-    <t>fortis_la_stock</t>
-  </si>
-  <si>
-    <t>Fortis LA</t>
-  </si>
-  <si>
-    <t>hk_slim_stock</t>
-  </si>
-  <si>
     <t>HK Slim Line</t>
   </si>
   <si>
-    <t>si_viper_mod1_stock</t>
-  </si>
-  <si>
-    <t>Strike Industries Viper MOD1 Stock</t>
-  </si>
-  <si>
-    <t>viper_rubber_pad</t>
-  </si>
-  <si>
-    <t>magpul_moe_carbine_stock</t>
-  </si>
-  <si>
     <t>MOE Carbine</t>
   </si>
   <si>
-    <t>magpul_moe_butt_pad</t>
-  </si>
-  <si>
-    <t>ar_tr2_stock</t>
-  </si>
-  <si>
-    <t>AR TR2</t>
-  </si>
-  <si>
-    <t>ar_tr2_pad</t>
-  </si>
-  <si>
-    <t>vltor_emod_stock</t>
-  </si>
-  <si>
     <t>VLtor Emod</t>
   </si>
   <si>
-    <t>emod_pad</t>
-  </si>
-  <si>
-    <t>magpul_prs_gen3_stock</t>
-  </si>
-  <si>
-    <t>Magpul PRS Gen3 Stock</t>
-  </si>
-  <si>
-    <t>prs_adjustable_piece</t>
-  </si>
-  <si>
-    <t>prs_gen3_buttpad</t>
-  </si>
-  <si>
-    <t>Magpul PRS Gen3 Buttpad</t>
-  </si>
-  <si>
-    <t>hera_arms_ccs_stock</t>
-  </si>
-  <si>
     <t>Hera Arms CSS</t>
   </si>
   <si>
-    <t>ak12_gen1_std_stock</t>
-  </si>
-  <si>
-    <t>Kalashnikov Concern AK-12 Gen 1</t>
-  </si>
-  <si>
-    <t>colt_m4ss_stock</t>
-  </si>
-  <si>
     <t>Colt M4SS</t>
   </si>
   <si>
-    <t>lmt_pad</t>
-  </si>
-  <si>
-    <t>lmt_sopmod</t>
-  </si>
-  <si>
-    <t>LMT Sopmod</t>
-  </si>
-  <si>
-    <t>brwnls_xm177_car</t>
-  </si>
-  <si>
-    <t>Brownells XM177 CAR</t>
-  </si>
-  <si>
-    <t>cf_rubber_buttpad</t>
-  </si>
-  <si>
-    <t>magpul_str_carbine_stock</t>
-  </si>
-  <si>
-    <t>Magpul STR Carbine</t>
-  </si>
-  <si>
-    <t>magpul_str_butt_pad</t>
-  </si>
-  <si>
-    <t>CURRENT</t>
-  </si>
-  <si>
-    <t>magazine_capacity</t>
-  </si>
-  <si>
-    <t>bullet_damage</t>
-  </si>
-  <si>
-    <t>bullet_velocity</t>
-  </si>
-  <si>
-    <t>fire_rate</t>
-  </si>
-  <si>
-    <t>strength score</t>
-  </si>
-  <si>
-    <t>irl weight</t>
-  </si>
-  <si>
-    <t>weight formula</t>
-  </si>
-  <si>
-    <t>irl price</t>
-  </si>
-  <si>
-    <t>price formula</t>
-  </si>
-  <si>
-    <t>UTG A2 Fixed</t>
-  </si>
-  <si>
-    <t>mdt_buttpad</t>
-  </si>
-  <si>
-    <t>MDT V5</t>
-  </si>
-  <si>
-    <t>Magpul UBR Gen2 Receiver Extension</t>
-  </si>
-  <si>
-    <t>Magpul UBR Gen2</t>
-  </si>
-  <si>
-    <t>Doublestar ACE M4 SOCOM</t>
-  </si>
-  <si>
-    <t>Doublestar ACE M4 SOCOM Buttpad</t>
-  </si>
-  <si>
-    <t>Viper Rubber Buttpad</t>
-  </si>
-  <si>
-    <t>Magpul MOE Carbine</t>
-  </si>
-  <si>
-    <t>AR TR2 Buttpad</t>
-  </si>
-  <si>
-    <t>VLTOR EMOD</t>
-  </si>
-  <si>
-    <t>EMOD Buttpad</t>
-  </si>
-  <si>
-    <t>Magpul PRS Gen3 Adjustment Piece</t>
-  </si>
-  <si>
-    <t>Hera Arms CCS</t>
-  </si>
-  <si>
-    <t>CF Rubber Buttpad</t>
-  </si>
-  <si>
-    <t>CURRENT (SUMMED)</t>
-  </si>
-  <si>
-    <t>Hera Arms CQR Gen2</t>
-  </si>
-  <si>
-    <t>magpul_moe_sl_k_carbine_stock</t>
-  </si>
-  <si>
-    <t>Magpul MOE SL-K Carbine</t>
-  </si>
-  <si>
-    <t>magpul_moe_sl_k_carbine_stock_buttpad</t>
-  </si>
-  <si>
-    <t>Magpul MOE SL-K Carbine Buttpad</t>
-  </si>
-  <si>
-    <t>Magpul STR Carbine Buttpad</t>
-  </si>
-  <si>
-    <t>Magpul MOE Carbine Buttpad</t>
-  </si>
-  <si>
-    <t>LMT Sopmod Buttpad</t>
-  </si>
-  <si>
-    <t>daniel_defense_collapsible_milspec_buttstock</t>
-  </si>
-  <si>
-    <t>Daniel Defense Collapsible Milspec Stock</t>
-  </si>
-  <si>
-    <t>daniel_defense_concave_buttpad</t>
-  </si>
-  <si>
-    <t>Daniel Defense Concave Buttpad</t>
-  </si>
-  <si>
-    <t>colt_607_car15_buffer_tube</t>
-  </si>
-  <si>
-    <t>Colt 607 CAR-15 Buffer Tube</t>
-  </si>
-  <si>
-    <t>colt_607_car15_stock</t>
-  </si>
-  <si>
-    <t>Colt 607 CAR-15 Stock</t>
-  </si>
-  <si>
-    <t>barrel_deviation</t>
-  </si>
-  <si>
-    <t>buck_barrel_deviation</t>
-  </si>
-  <si>
-    <t>troy_m7a1_pdw_extendable_stock</t>
-  </si>
-  <si>
-    <t>Troy M7A1 PDW Extendable Stock</t>
-  </si>
-  <si>
-    <t>troy_m7a1_pdw_base_stock</t>
-  </si>
-  <si>
-    <t>Troy M7A1 PDW Base</t>
+    <t>hart_m4a1_receiver_endplate</t>
+  </si>
+  <si>
+    <t>Hart M4A1 Receiver Endplate</t>
+  </si>
+  <si>
+    <t>hart_607_car15_buffer_tube</t>
+  </si>
+  <si>
+    <t>Hart 607 CAR-15 Buffer Tube</t>
+  </si>
+  <si>
+    <t>hart_607_car15_stock</t>
+  </si>
+  <si>
+    <t>Hart 607 CAR-15 Stock</t>
+  </si>
+  <si>
+    <t>leopard_atg_model_15_fixed_a2_ar15_stock</t>
+  </si>
+  <si>
+    <t>mcs_lss_stock_adapter</t>
+  </si>
+  <si>
+    <t>mcs_v5_skeleton_rifle_stock</t>
+  </si>
+  <si>
+    <t>mcs_v5_skeleton_rifle_stock_short</t>
+  </si>
+  <si>
+    <t>mcs_buttpad</t>
+  </si>
+  <si>
+    <t>magtap_ubr_gen2_buffer</t>
+  </si>
+  <si>
+    <t>hart_a2_buffer</t>
+  </si>
+  <si>
+    <t>Hart A2</t>
+  </si>
+  <si>
+    <t>magtap_prs_gen2_stock</t>
+  </si>
+  <si>
+    <t>hart_m4a1_castlenut</t>
+  </si>
+  <si>
+    <t>Hart M4A1 Castle Nut</t>
+  </si>
+  <si>
+    <t>starsurp_starsurp_apex_m4_socom_gen4_stock</t>
+  </si>
+  <si>
+    <t>Starsurp ACE M4 SOCOM</t>
+  </si>
+  <si>
+    <t>starsurp_starsurp_apex_0.5_recoil_pad</t>
+  </si>
+  <si>
+    <t>Starsurp ACE M4 SOCOM Buttpad</t>
+  </si>
+  <si>
+    <t>hart_buffer_tube</t>
+  </si>
+  <si>
+    <t>Hart</t>
+  </si>
+  <si>
+    <t>validus_la_stock</t>
+  </si>
+  <si>
+    <t>kf_416_slim_line_stock</t>
+  </si>
+  <si>
+    <t>KF416 Slim Line</t>
+  </si>
+  <si>
+    <t>magtap_moe_carbine_stock</t>
+  </si>
+  <si>
+    <t>magtap_moe_butt_pad</t>
+  </si>
+  <si>
+    <t>vyctor_emod_stock</t>
+  </si>
+  <si>
+    <t>magtap_prs_gen3_stock</t>
+  </si>
+  <si>
+    <t>hart_m4ss_stock</t>
+  </si>
+  <si>
+    <t>Hart M4SS</t>
+  </si>
+  <si>
+    <t>whtnls_xm177_car</t>
+  </si>
+  <si>
+    <t>magtap_str_carbine_stock</t>
+  </si>
+  <si>
+    <t>magtap_str_butt_pad</t>
+  </si>
+  <si>
+    <t>magtap_moe_sl_k_carbine_stock</t>
+  </si>
+  <si>
+    <t>magtap_moe_sl_k_carbine_stock_buttpad</t>
+  </si>
+  <si>
+    <t>axtell_defense_collapsible_milspec_buttstock</t>
+  </si>
+  <si>
+    <t>axtell_defense_concave_buttpad</t>
   </si>
 </sst>
 </file>
@@ -422,135 +431,99 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="18"/>
       <color theme="3"/>
       <name val="Calibri Light"/>
-      <family val="2"/>
-      <scheme val="major"/>
     </font>
     <font>
       <b/>
       <sz val="15"/>
       <color theme="3"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="13"/>
       <color theme="3"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="3"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C5700"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
@@ -602,13 +575,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
+        <fgColor theme="4" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
+        <fgColor theme="4" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -625,13 +598,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
+        <fgColor theme="5" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
+        <fgColor theme="5" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -648,13 +621,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
+        <fgColor theme="6" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
+        <fgColor theme="6" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -671,13 +644,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor theme="7" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
+        <fgColor theme="7" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -694,13 +667,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
+        <fgColor theme="8" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
+        <fgColor theme="8" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -717,13 +690,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
+        <fgColor theme="9" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
+        <fgColor theme="9" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -756,7 +729,7 @@
       <right/>
       <top/>
       <bottom style="thick">
-        <color theme="4" tint="0.499984740745262"/>
+        <color theme="4" tint="0.49995422223578601"/>
       </bottom>
       <diagonal/>
     </border>
@@ -898,48 +871,48 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="19" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="20% - Accent2" xfId="23" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="20% - Accent3" xfId="27" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="20% - Accent4" xfId="31" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="20% - Accent5" xfId="35" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="20% - Accent6" xfId="39" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="40% - Accent1" xfId="20" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="40% - Accent2" xfId="24" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="40% - Accent3" xfId="28" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="40% - Accent4" xfId="32" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="40% - Accent5" xfId="36" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
+    <cellStyle name="40% - Accent6" xfId="40" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
+    <cellStyle name="60% - Accent1" xfId="21" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
+    <cellStyle name="60% - Accent2" xfId="25" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
+    <cellStyle name="60% - Accent3" xfId="29" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
+    <cellStyle name="60% - Accent4" xfId="33" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
+    <cellStyle name="60% - Accent5" xfId="37" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="60% - Accent6" xfId="41" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
+    <cellStyle name="Accent1" xfId="18" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
+    <cellStyle name="Accent2" xfId="22" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
+    <cellStyle name="Accent3" xfId="26" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
+    <cellStyle name="Accent4" xfId="30" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
+    <cellStyle name="Accent5" xfId="34" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
+    <cellStyle name="Accent6" xfId="38" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
+    <cellStyle name="Bad" xfId="7" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
+    <cellStyle name="Calculation" xfId="11" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
+    <cellStyle name="Check Cell" xfId="13" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
+    <cellStyle name="Explanatory Text" xfId="16" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
+    <cellStyle name="Good" xfId="6" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
+    <cellStyle name="Heading 1" xfId="2" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
+    <cellStyle name="Heading 2" xfId="3" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
+    <cellStyle name="Heading 3" xfId="4" xr:uid="{00000000-0005-0000-0000-00001F000000}"/>
+    <cellStyle name="Heading 4" xfId="5" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
+    <cellStyle name="Input" xfId="9" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
+    <cellStyle name="Linked Cell" xfId="12" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
+    <cellStyle name="Neutral" xfId="8" xr:uid="{00000000-0005-0000-0000-000023000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Note" xfId="15" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
+    <cellStyle name="Output" xfId="10" xr:uid="{00000000-0005-0000-0000-000026000000}"/>
+    <cellStyle name="Title" xfId="1" xr:uid="{00000000-0005-0000-0000-000027000000}"/>
+    <cellStyle name="Total" xfId="17" xr:uid="{00000000-0005-0000-0000-000028000000}"/>
+    <cellStyle name="Warning Text" xfId="14" xr:uid="{00000000-0005-0000-0000-000029000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -995,110 +968,16 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office 2013 - 2022">
@@ -1110,23 +989,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
                 <a:lumMod val="110000"/>
                 <a:satMod val="105000"/>
-                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="103000"/>
-                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="109000"/>
-                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1136,23 +1015,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
                 <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
                 <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
                 <a:lumMod val="99000"/>
                 <a:satMod val="120000"/>
-                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1160,26 +1039,23 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="19050">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -1214,17 +1090,17 @@
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
+                <a:satMod val="150000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
@@ -1241,11 +1117,6 @@
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
@@ -1260,71 +1131,71 @@
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
-        <v>78</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G2" t="s">
-        <v>79</v>
+        <v>7</v>
       </c>
       <c r="H2" t="s">
-        <v>120</v>
+        <v>8</v>
       </c>
       <c r="I2" t="s">
-        <v>80</v>
+        <v>9</v>
       </c>
       <c r="J2" t="s">
-        <v>81</v>
+        <v>10</v>
       </c>
       <c r="K2" t="s">
-        <v>121</v>
+        <v>11</v>
       </c>
       <c r="L2" t="s">
-        <v>82</v>
+        <v>12</v>
       </c>
       <c r="M2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="N2" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="P2" t="s">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="Q2" t="s">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="R2" t="s">
-        <v>86</v>
+        <v>17</v>
       </c>
       <c r="S2" t="s">
-        <v>87</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -1349,8 +1220,8 @@
         <v>19</v>
       </c>
       <c r="Q3">
-        <f>P3*0.025</f>
-        <v>0.47500000000000003</v>
+        <f>P3*0.024</f>
+        <v>0.45600000000000002</v>
       </c>
       <c r="R3">
         <v>129</v>
@@ -1358,10 +1229,10 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -1379,20 +1250,20 @@
         <v>0</v>
       </c>
       <c r="N4">
-        <f t="shared" ref="N4:N67" si="0">C4-(D4*20)-(E4*0.8)-(F4*0.6)-(H4*5)</f>
+        <f t="shared" ref="N4:N56" si="0">C4-(D4*20)-(E4*0.8)-(F4*0.6)-(H4*5)</f>
         <v>1.4</v>
       </c>
       <c r="Q4">
-        <f t="shared" ref="Q4:Q54" si="1">P4*0.025</f>
+        <f t="shared" ref="Q4:Q54" si="1">P4*0.024</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>90</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>91</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -1412,15 +1283,15 @@
       </c>
       <c r="Q5">
         <f t="shared" si="1"/>
-        <v>1.0000000000000002E-2</v>
+        <v>9.6000000000000009E-3</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>116</v>
+        <v>92</v>
       </c>
       <c r="B6" t="s">
-        <v>117</v>
+        <v>93</v>
       </c>
       <c r="C6">
         <v>-2</v>
@@ -1448,10 +1319,10 @@
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="B7" t="s">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="C7">
         <v>16</v>
@@ -1479,10 +1350,10 @@
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>124</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>125</v>
+        <v>24</v>
       </c>
       <c r="C8">
         <v>-2</v>
@@ -1500,15 +1371,15 @@
         <v>1000</v>
       </c>
       <c r="N8">
-        <f>C8-(D8*20)-(E8*0.8)-(F8*0.6)-(H8*5)</f>
+        <f t="shared" si="0"/>
         <v>-4.4000000000000004</v>
       </c>
       <c r="P8">
         <v>14</v>
       </c>
       <c r="Q8">
-        <f>P8*0.025</f>
-        <v>0.35000000000000003</v>
+        <f t="shared" si="1"/>
+        <v>0.33600000000000002</v>
       </c>
       <c r="R8">
         <v>479.99</v>
@@ -1526,10 +1397,10 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>122</v>
+        <v>25</v>
       </c>
       <c r="B10" t="s">
-        <v>123</v>
+        <v>26</v>
       </c>
       <c r="C10">
         <v>21</v>
@@ -1557,10 +1428,10 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>96</v>
       </c>
       <c r="B11" t="s">
-        <v>88</v>
+        <v>27</v>
       </c>
       <c r="C11">
         <v>11</v>
@@ -1586,7 +1457,7 @@
       </c>
       <c r="Q11">
         <f t="shared" si="1"/>
-        <v>0.625</v>
+        <v>0.6</v>
       </c>
       <c r="R11">
         <v>79.97</v>
@@ -1594,10 +1465,10 @@
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>97</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="C12">
         <v>-1</v>
@@ -1619,10 +1490,10 @@
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>98</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="C13">
         <v>22</v>
@@ -1651,7 +1522,7 @@
       </c>
       <c r="Q13">
         <f t="shared" si="1"/>
-        <v>0.79200000000000004</v>
+        <v>0.76032</v>
       </c>
       <c r="R13">
         <v>399.95</v>
@@ -1659,10 +1530,10 @@
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C14">
         <v>22</v>
@@ -1691,7 +1562,7 @@
       </c>
       <c r="Q14">
         <f t="shared" si="1"/>
-        <v>0.79200000000000004</v>
+        <v>0.76032</v>
       </c>
       <c r="R14">
         <v>389.95</v>
@@ -1699,10 +1570,10 @@
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="B15" t="s">
-        <v>90</v>
+        <v>31</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -1730,10 +1601,10 @@
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>101</v>
       </c>
       <c r="B16" t="s">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="C16">
         <v>-1</v>
@@ -1747,15 +1618,12 @@
       <c r="F16">
         <v>-2</v>
       </c>
-      <c r="H16">
-        <v>-0.05</v>
-      </c>
       <c r="M16">
         <v>400</v>
       </c>
       <c r="N16">
         <f t="shared" si="0"/>
-        <v>-1.55</v>
+        <v>-1.8</v>
       </c>
       <c r="Q16">
         <f t="shared" si="1"/>
@@ -1764,10 +1632,10 @@
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="B17" t="s">
-        <v>92</v>
+        <v>34</v>
       </c>
       <c r="C17">
         <v>14</v>
@@ -1779,21 +1647,21 @@
         <v>-14</v>
       </c>
       <c r="F17">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="M17">
         <v>700</v>
       </c>
       <c r="N17">
         <f t="shared" si="0"/>
-        <v>23</v>
+        <v>24.2</v>
       </c>
       <c r="P17">
         <v>21.3</v>
       </c>
       <c r="Q17">
         <f t="shared" si="1"/>
-        <v>0.53250000000000008</v>
+        <v>0.51119999999999999</v>
       </c>
       <c r="R17">
         <v>199.95</v>
@@ -1801,10 +1669,10 @@
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>102</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>103</v>
       </c>
       <c r="C18">
         <v>-2</v>
@@ -1818,15 +1686,12 @@
       <c r="F18">
         <v>-1</v>
       </c>
-      <c r="H18">
-        <v>-0.05</v>
-      </c>
       <c r="M18">
         <v>300</v>
       </c>
       <c r="N18">
         <f t="shared" si="0"/>
-        <v>-3.35</v>
+        <v>-3.6</v>
       </c>
       <c r="Q18">
         <f t="shared" si="1"/>
@@ -1838,36 +1703,39 @@
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>104</v>
       </c>
       <c r="B19" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C19">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D19">
         <v>0.38</v>
       </c>
       <c r="E19">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="F19">
-        <v>-5</v>
+        <v>-15</v>
+      </c>
+      <c r="H19">
+        <v>-0.05</v>
       </c>
       <c r="M19">
         <v>1200</v>
       </c>
       <c r="N19">
         <f t="shared" si="0"/>
-        <v>19.8</v>
+        <v>24.85</v>
       </c>
       <c r="P19">
         <v>31.4</v>
       </c>
       <c r="Q19">
         <f t="shared" si="1"/>
-        <v>0.78500000000000003</v>
+        <v>0.75359999999999994</v>
       </c>
       <c r="R19">
         <v>208.25</v>
@@ -1875,13 +1743,13 @@
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="B20" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C20">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D20">
         <v>0.16</v>
@@ -1890,21 +1758,21 @@
         <v>-7</v>
       </c>
       <c r="F20">
-        <v>-8</v>
+        <v>-10</v>
       </c>
       <c r="M20">
         <v>1000</v>
       </c>
       <c r="N20">
         <f t="shared" si="0"/>
-        <v>22.200000000000003</v>
+        <v>24.400000000000002</v>
       </c>
       <c r="P20">
         <v>15.2</v>
       </c>
       <c r="Q20">
         <f t="shared" si="1"/>
-        <v>0.38</v>
+        <v>0.36480000000000001</v>
       </c>
       <c r="R20">
         <v>59.9</v>
@@ -1912,10 +1780,10 @@
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>31</v>
+        <v>105</v>
       </c>
       <c r="B21" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -1935,7 +1803,7 @@
       </c>
       <c r="Q21">
         <f t="shared" si="1"/>
-        <v>1.4999999999999999E-2</v>
+        <v>1.44E-2</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
@@ -1950,10 +1818,10 @@
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>33</v>
+        <v>107</v>
       </c>
       <c r="B23" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="C23">
         <v>14</v>
@@ -1979,7 +1847,7 @@
       </c>
       <c r="Q23">
         <f t="shared" si="1"/>
-        <v>0.47500000000000003</v>
+        <v>0.45600000000000002</v>
       </c>
       <c r="R23">
         <v>244.99</v>
@@ -1987,10 +1855,10 @@
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>35</v>
+        <v>109</v>
       </c>
       <c r="B24" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="C24">
         <v>2</v>
@@ -2018,10 +1886,10 @@
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B25" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C25">
         <v>18</v>
@@ -2047,21 +1915,21 @@
       </c>
       <c r="Q25">
         <f t="shared" si="1"/>
-        <v>0.36000000000000004</v>
+        <v>0.34560000000000002</v>
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C26">
         <v>-1</v>
       </c>
       <c r="D26">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="E26">
         <v>-1</v>
@@ -2069,22 +1937,19 @@
       <c r="F26">
         <v>-1</v>
       </c>
-      <c r="H26">
-        <v>0</v>
-      </c>
       <c r="M26">
         <v>600</v>
       </c>
       <c r="N26">
         <f t="shared" si="0"/>
-        <v>-1.8000000000000003</v>
+        <v>-2.1999999999999997</v>
       </c>
       <c r="P26">
-        <v>3.8</v>
+        <v>6.8</v>
       </c>
       <c r="Q26">
         <f t="shared" si="1"/>
-        <v>9.5000000000000001E-2</v>
+        <v>0.16320000000000001</v>
       </c>
       <c r="R26">
         <v>52.95</v>
@@ -2092,10 +1957,10 @@
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>40</v>
+        <v>111</v>
       </c>
       <c r="B27" t="s">
-        <v>41</v>
+        <v>112</v>
       </c>
       <c r="C27">
         <v>-2</v>
@@ -2107,24 +1972,21 @@
         <v>-2</v>
       </c>
       <c r="F27">
-        <v>-1</v>
-      </c>
-      <c r="H27">
-        <v>-0.1</v>
+        <v>-2</v>
       </c>
       <c r="M27">
         <v>0</v>
       </c>
       <c r="N27">
         <f t="shared" si="0"/>
-        <v>-2.2999999999999998</v>
+        <v>-2.2000000000000002</v>
       </c>
       <c r="P27">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q27">
         <f t="shared" si="1"/>
-        <v>0.15000000000000002</v>
+        <v>0.16800000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
@@ -2139,10 +2001,10 @@
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>113</v>
+      </c>
+      <c r="B29" t="s">
         <v>42</v>
-      </c>
-      <c r="B29" t="s">
-        <v>43</v>
       </c>
       <c r="C29">
         <v>17</v>
@@ -2168,7 +2030,7 @@
       </c>
       <c r="Q29">
         <f t="shared" si="1"/>
-        <v>0.39500000000000002</v>
+        <v>0.37920000000000004</v>
       </c>
       <c r="R29">
         <v>349.95</v>
@@ -2176,10 +2038,10 @@
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>44</v>
+        <v>114</v>
       </c>
       <c r="B30" t="s">
-        <v>45</v>
+        <v>115</v>
       </c>
       <c r="C30">
         <v>16</v>
@@ -2205,7 +2067,7 @@
       </c>
       <c r="Q30">
         <f t="shared" si="1"/>
-        <v>0.32500000000000001</v>
+        <v>0.312</v>
       </c>
       <c r="R30">
         <v>249.95</v>
@@ -2213,10 +2075,10 @@
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B31" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C31">
         <v>18</v>
@@ -2242,7 +2104,7 @@
       </c>
       <c r="Q31">
         <f t="shared" si="1"/>
-        <v>0.16500000000000001</v>
+        <v>0.15839999999999999</v>
       </c>
       <c r="R31">
         <v>45.95</v>
@@ -2250,10 +2112,10 @@
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B32" t="s">
-        <v>95</v>
+        <v>46</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -2281,10 +2143,10 @@
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>49</v>
+        <v>116</v>
       </c>
       <c r="B33" t="s">
-        <v>96</v>
+        <v>47</v>
       </c>
       <c r="C33">
         <v>17</v>
@@ -2310,7 +2172,7 @@
       </c>
       <c r="Q33">
         <f t="shared" si="1"/>
-        <v>0.21000000000000002</v>
+        <v>0.2016</v>
       </c>
       <c r="R33">
         <v>44.95</v>
@@ -2318,10 +2180,10 @@
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>51</v>
+        <v>117</v>
       </c>
       <c r="B34" t="s">
-        <v>110</v>
+        <v>48</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -2349,10 +2211,10 @@
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B35" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C35">
         <v>16</v>
@@ -2378,7 +2240,7 @@
       </c>
       <c r="Q35">
         <f t="shared" si="1"/>
-        <v>0.38750000000000001</v>
+        <v>0.372</v>
       </c>
       <c r="R35">
         <v>250</v>
@@ -2386,10 +2248,10 @@
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B36" t="s">
-        <v>97</v>
+        <v>52</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -2417,10 +2279,10 @@
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="B37" t="s">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="C37">
         <v>14</v>
@@ -2446,7 +2308,7 @@
       </c>
       <c r="Q37">
         <f t="shared" si="1"/>
-        <v>0.35000000000000003</v>
+        <v>0.33600000000000002</v>
       </c>
       <c r="R37">
         <v>197.95</v>
@@ -2454,10 +2316,10 @@
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B38" t="s">
-        <v>99</v>
+        <v>55</v>
       </c>
       <c r="C38">
         <v>1</v>
@@ -2485,13 +2347,13 @@
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>58</v>
+        <v>119</v>
       </c>
       <c r="B39" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C39">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D39">
         <v>0.33</v>
@@ -2500,7 +2362,7 @@
         <v>-4</v>
       </c>
       <c r="F39">
-        <v>-3</v>
+        <v>-16</v>
       </c>
       <c r="H39">
         <v>-0.05</v>
@@ -2510,14 +2372,14 @@
       </c>
       <c r="N39">
         <f t="shared" si="0"/>
-        <v>18.649999999999999</v>
+        <v>24.449999999999996</v>
       </c>
       <c r="P39">
         <v>27.8</v>
       </c>
       <c r="Q39">
         <f t="shared" si="1"/>
-        <v>0.69500000000000006</v>
+        <v>0.66720000000000002</v>
       </c>
       <c r="R39">
         <v>259.95</v>
@@ -2525,10 +2387,10 @@
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B40" t="s">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="C40">
         <v>0</v>
@@ -2550,10 +2412,10 @@
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B41" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C41">
         <v>1</v>
@@ -2581,10 +2443,10 @@
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B42" t="s">
-        <v>101</v>
+        <v>62</v>
       </c>
       <c r="C42">
         <v>15</v>
@@ -2610,7 +2472,7 @@
       </c>
       <c r="Q42">
         <f t="shared" si="1"/>
-        <v>0.23750000000000002</v>
+        <v>0.22800000000000001</v>
       </c>
       <c r="R42">
         <v>59.9</v>
@@ -2618,10 +2480,10 @@
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B43" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C43">
         <v>16</v>
@@ -2647,15 +2509,15 @@
       </c>
       <c r="Q43">
         <f t="shared" si="1"/>
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>67</v>
+        <v>120</v>
       </c>
       <c r="B44" t="s">
-        <v>68</v>
+        <v>121</v>
       </c>
       <c r="C44">
         <v>16</v>
@@ -2681,15 +2543,15 @@
       </c>
       <c r="Q44">
         <f t="shared" si="1"/>
-        <v>0.2</v>
+        <v>0.192</v>
       </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B45" t="s">
-        <v>111</v>
+        <v>66</v>
       </c>
       <c r="C45">
         <v>1</v>
@@ -2717,10 +2579,10 @@
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B46" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C46">
         <v>18</v>
@@ -2746,7 +2608,7 @@
       </c>
       <c r="Q46">
         <f t="shared" si="1"/>
-        <v>0.31000000000000005</v>
+        <v>0.29760000000000003</v>
       </c>
       <c r="R46">
         <v>209</v>
@@ -2754,10 +2616,10 @@
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>72</v>
+        <v>122</v>
       </c>
       <c r="B47" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C47">
         <v>16</v>
@@ -2783,7 +2645,7 @@
       </c>
       <c r="Q47">
         <f t="shared" si="1"/>
-        <v>0.11499999999999999</v>
+        <v>0.1104</v>
       </c>
       <c r="R47">
         <v>50</v>
@@ -2791,10 +2653,10 @@
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B48" t="s">
-        <v>102</v>
+        <v>71</v>
       </c>
       <c r="C48">
         <v>1</v>
@@ -2820,15 +2682,15 @@
       </c>
       <c r="Q48">
         <f t="shared" si="1"/>
-        <v>2.5000000000000001E-2</v>
+        <v>2.4E-2</v>
       </c>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>75</v>
+        <v>123</v>
       </c>
       <c r="B49" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C49">
         <v>17</v>
@@ -2854,7 +2716,7 @@
       </c>
       <c r="Q49">
         <f t="shared" si="1"/>
-        <v>0.315</v>
+        <v>0.3024</v>
       </c>
       <c r="R49">
         <v>84.95</v>
@@ -2862,10 +2724,10 @@
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>77</v>
+        <v>124</v>
       </c>
       <c r="B50" t="s">
-        <v>109</v>
+        <v>73</v>
       </c>
       <c r="C50">
         <v>1</v>
@@ -2893,10 +2755,10 @@
     </row>
     <row r="51" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="B51" t="s">
-        <v>106</v>
+        <v>74</v>
       </c>
       <c r="C51">
         <v>18</v>
@@ -2922,7 +2784,7 @@
       </c>
       <c r="Q51">
         <f t="shared" si="1"/>
-        <v>0.19500000000000001</v>
+        <v>0.18720000000000001</v>
       </c>
       <c r="R51">
         <v>44.95</v>
@@ -2930,10 +2792,10 @@
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="B52" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
       <c r="C52">
         <v>1</v>
@@ -2961,10 +2823,10 @@
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="B53" t="s">
-        <v>113</v>
+        <v>76</v>
       </c>
       <c r="C53">
         <v>16</v>
@@ -2990,7 +2852,7 @@
       </c>
       <c r="Q53">
         <f t="shared" si="1"/>
-        <v>0.2</v>
+        <v>0.192</v>
       </c>
       <c r="R53">
         <v>82</v>
@@ -2998,10 +2860,10 @@
     </row>
     <row r="54" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="B54" t="s">
-        <v>115</v>
+        <v>77</v>
       </c>
       <c r="C54">
         <v>1</v>
@@ -3035,7 +2897,7 @@
     </row>
     <row r="56" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="N56">
         <f t="shared" si="0"/>
@@ -3044,10 +2906,10 @@
     </row>
     <row r="57" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
-        <v>104</v>
+        <v>79</v>
       </c>
       <c r="C57">
-        <f t="shared" ref="C57:M57" si="2">C4+C3</f>
+        <f t="shared" ref="C57:S57" si="2">C4+C3</f>
         <v>11</v>
       </c>
       <c r="D57">
@@ -3091,23 +2953,23 @@
         <v>1500</v>
       </c>
       <c r="N57">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>17</v>
       </c>
       <c r="O57">
-        <f>O4+O3</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P57">
-        <f>P4+P3</f>
+        <f t="shared" si="2"/>
         <v>19</v>
       </c>
       <c r="Q57">
-        <f>P57*0.015+0.15</f>
-        <v>0.43499999999999994</v>
+        <f t="shared" si="2"/>
+        <v>0.45600000000000002</v>
       </c>
       <c r="R57">
-        <f>R4+R3</f>
+        <f t="shared" si="2"/>
         <v>129</v>
       </c>
       <c r="S57">
@@ -3117,10 +2979,10 @@
     </row>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="C58">
-        <f t="shared" ref="C58:M58" si="4">C6+C7</f>
+        <f t="shared" ref="C58:R58" si="4">C6+C7</f>
         <v>14</v>
       </c>
       <c r="D58">
@@ -3164,64 +3026,64 @@
         <v>1000</v>
       </c>
       <c r="N58">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="N57:N67" si="5">C58-(D58*20)-(E58*0.8)-(F58*0.6)-(H58*5)</f>
         <v>23</v>
       </c>
       <c r="Q58">
-        <f t="shared" ref="Q58:Q82" si="5">P58*0.015+0.15</f>
+        <f t="shared" ref="Q58:Q82" si="6">P58*0.015+0.15</f>
         <v>0.15</v>
       </c>
     </row>
     <row r="59" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
-        <v>13</v>
+        <v>81</v>
       </c>
       <c r="C59">
-        <f t="shared" ref="C59:M59" si="6">C10+C8+C5</f>
+        <f t="shared" ref="C59:R59" si="7">C10+C8+C5</f>
         <v>19</v>
       </c>
       <c r="D59">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.28000000000000003</v>
       </c>
       <c r="E59">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-6</v>
       </c>
       <c r="F59">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-7</v>
       </c>
       <c r="G59">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="H59">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="I59">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J59">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K59">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="L59">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="M59">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1800</v>
       </c>
       <c r="N59">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>22.4</v>
       </c>
       <c r="P59">
@@ -3229,7 +3091,7 @@
         <v>14.4</v>
       </c>
       <c r="Q59">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.36599999999999999</v>
       </c>
       <c r="R59">
@@ -3243,54 +3105,54 @@
     </row>
     <row r="60" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
-        <v>15</v>
+        <v>82</v>
       </c>
       <c r="C60">
-        <f t="shared" ref="C60:M60" si="7">C11+C5</f>
+        <f t="shared" ref="C60:R60" si="8">C11+C5</f>
         <v>11</v>
       </c>
       <c r="D60">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.45</v>
       </c>
       <c r="E60">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-12</v>
       </c>
       <c r="F60">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-18</v>
       </c>
       <c r="G60">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="H60">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I60">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J60">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="K60">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="L60">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M60">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>700</v>
       </c>
       <c r="N60">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>22.4</v>
       </c>
       <c r="P60">
@@ -3298,7 +3160,7 @@
         <v>25.4</v>
       </c>
       <c r="Q60">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.53099999999999992</v>
       </c>
       <c r="R60">
@@ -3312,54 +3174,54 @@
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="C61">
-        <f t="shared" ref="C61:M61" si="8">C13+C12+C5+C15</f>
+        <f t="shared" ref="C61:R61" si="9">C13+C12+C5+C15</f>
         <v>22</v>
       </c>
       <c r="D61">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0.42</v>
       </c>
       <c r="E61">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-1</v>
       </c>
       <c r="F61">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-1</v>
       </c>
       <c r="G61">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="H61">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-0.05</v>
       </c>
       <c r="I61">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J61">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="K61">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="L61">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="M61">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1300</v>
       </c>
       <c r="N61">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>15.25</v>
       </c>
       <c r="P61">
@@ -3367,7 +3229,7 @@
         <v>32.08</v>
       </c>
       <c r="Q61">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.63119999999999998</v>
       </c>
       <c r="R61">
@@ -3381,54 +3243,54 @@
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C62">
-        <f t="shared" ref="C62:M62" si="9">C14+C12+C5+C15</f>
+        <f t="shared" ref="C62:M62" si="10">C14+C12+C5+C15</f>
         <v>22</v>
       </c>
       <c r="D62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.39999999999999997</v>
       </c>
       <c r="E62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-1</v>
       </c>
       <c r="F62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-1</v>
       </c>
       <c r="G62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="H62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-0.05</v>
       </c>
       <c r="I62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="K62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="L62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="M62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1300</v>
       </c>
       <c r="N62">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>15.65</v>
       </c>
       <c r="P62">
@@ -3436,7 +3298,7 @@
         <v>32.08</v>
       </c>
       <c r="Q62">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.63119999999999998</v>
       </c>
       <c r="R62">
@@ -3450,62 +3312,62 @@
     </row>
     <row r="63" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="C63">
-        <f t="shared" ref="C63:M63" si="10">C17+C16+C5</f>
+        <f t="shared" ref="C63:N63" si="11">C17+C16+C5</f>
         <v>13</v>
       </c>
       <c r="D63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0.44</v>
       </c>
       <c r="E63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-15</v>
       </c>
       <c r="F63">
-        <f t="shared" si="10"/>
-        <v>-8</v>
+        <f t="shared" si="11"/>
+        <v>-10</v>
       </c>
       <c r="G63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="H63">
-        <f t="shared" si="10"/>
-        <v>-0.05</v>
+        <f t="shared" si="11"/>
+        <v>0</v>
       </c>
       <c r="I63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="K63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="L63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="M63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>1100</v>
       </c>
       <c r="N63">
-        <f t="shared" si="0"/>
-        <v>21.25</v>
+        <f t="shared" si="5"/>
+        <v>22.2</v>
       </c>
       <c r="P63">
         <f>P17+P16+P5</f>
         <v>21.7</v>
       </c>
       <c r="Q63">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.47549999999999992</v>
       </c>
       <c r="R63">
@@ -3519,62 +3381,62 @@
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C64">
-        <f t="shared" ref="C64:M64" si="11">C19+C18+C5</f>
-        <v>20</v>
+        <f t="shared" ref="C64:N64" si="12">C19+C18+C5</f>
+        <v>18</v>
       </c>
       <c r="D64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.54</v>
       </c>
       <c r="E64">
-        <f t="shared" si="11"/>
-        <v>-4</v>
+        <f t="shared" si="12"/>
+        <v>-5</v>
       </c>
       <c r="F64">
-        <f t="shared" si="11"/>
-        <v>-6</v>
+        <f t="shared" si="12"/>
+        <v>-16</v>
       </c>
       <c r="G64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="H64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-0.05</v>
       </c>
       <c r="I64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="J64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="K64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="L64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="M64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1500</v>
       </c>
       <c r="N64">
-        <f t="shared" si="0"/>
-        <v>16.25</v>
+        <f t="shared" si="12"/>
+        <v>21.05</v>
       </c>
       <c r="P64">
         <f>P19+P18+P5</f>
         <v>31.799999999999997</v>
       </c>
       <c r="Q64">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.62699999999999989</v>
       </c>
       <c r="R64">
@@ -3588,62 +3450,62 @@
     </row>
     <row r="65" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B65" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C65">
-        <f t="shared" ref="C65:M65" si="12">C20+C18+C5</f>
-        <v>13</v>
+        <f t="shared" ref="C65:N65" si="13">C20+C18+C5</f>
+        <v>14</v>
       </c>
       <c r="D65">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0.32</v>
       </c>
       <c r="E65">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-8</v>
       </c>
       <c r="F65">
-        <f t="shared" si="12"/>
-        <v>-9</v>
+        <f t="shared" si="13"/>
+        <v>-11</v>
       </c>
       <c r="G65">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="H65">
-        <f t="shared" si="12"/>
-        <v>-0.05</v>
+        <f t="shared" si="13"/>
+        <v>0</v>
       </c>
       <c r="I65">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="J65">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="K65">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L65">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="M65">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1300</v>
       </c>
       <c r="N65">
-        <f t="shared" si="0"/>
-        <v>18.649999999999999</v>
+        <f t="shared" si="13"/>
+        <v>20.6</v>
       </c>
       <c r="P65">
         <f>P20+P18+P5</f>
         <v>15.6</v>
       </c>
       <c r="Q65">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.38400000000000001</v>
       </c>
       <c r="R65">
@@ -3657,54 +3519,54 @@
     </row>
     <row r="66" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B66" t="s">
-        <v>34</v>
+        <v>84</v>
       </c>
       <c r="C66">
-        <f t="shared" ref="C66:M66" si="13">C24+C23+C21+C5</f>
+        <f t="shared" ref="C66:M66" si="14">C24+C23+C21+C5</f>
         <v>16</v>
       </c>
       <c r="D66">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0.38</v>
       </c>
       <c r="E66">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-10</v>
       </c>
       <c r="F66">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-10</v>
       </c>
       <c r="G66">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="H66">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="I66">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="J66">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="K66">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="L66">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="M66">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1000</v>
       </c>
       <c r="N66">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>22.4</v>
       </c>
       <c r="P66">
@@ -3712,7 +3574,7 @@
         <v>20</v>
       </c>
       <c r="Q66">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.44999999999999996</v>
       </c>
       <c r="R66">
@@ -3726,54 +3588,54 @@
     </row>
     <row r="67" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C67">
-        <f t="shared" ref="C67:M67" si="14">C25+C21+C5</f>
+        <f t="shared" ref="C67:M67" si="15">C25+C21+C5</f>
         <v>18</v>
       </c>
       <c r="D67">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0.31000000000000005</v>
       </c>
       <c r="E67">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>-4</v>
       </c>
       <c r="F67">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>-4</v>
       </c>
       <c r="G67">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="H67">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="I67">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="J67">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="K67">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="L67">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="M67">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>500</v>
       </c>
       <c r="N67">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>17.399999999999999</v>
       </c>
       <c r="P67">
@@ -3781,7 +3643,7 @@
         <v>15.4</v>
       </c>
       <c r="Q67">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.38100000000000001</v>
       </c>
       <c r="R67">
@@ -3795,63 +3657,63 @@
     </row>
     <row r="68" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B68" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C68">
-        <f t="shared" ref="C68:M68" si="15">C29+C26+C21+C5</f>
+        <f t="shared" ref="C68:M68" si="16">C29+C26+C21+C5</f>
         <v>16</v>
       </c>
       <c r="D68">
-        <f t="shared" si="15"/>
-        <v>0.34</v>
+        <f t="shared" si="16"/>
+        <v>0.36000000000000004</v>
       </c>
       <c r="E68">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-13</v>
       </c>
       <c r="F68">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-7</v>
       </c>
       <c r="G68">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="H68">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="I68">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="J68">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="K68">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="L68">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="M68">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>1500</v>
       </c>
       <c r="N68">
-        <f t="shared" ref="N68:N82" si="16">C68-(D68*20)-(E68*0.8)-(F68*0.6)-(H68*5)</f>
-        <v>23.8</v>
+        <f t="shared" ref="N68:N82" si="17">C68-(D68*20)-(E68*0.8)-(F68*0.6)-(H68*5)</f>
+        <v>23.4</v>
       </c>
       <c r="P68">
         <f>P29+P26+P21+P5</f>
-        <v>20.6</v>
+        <v>23.6</v>
       </c>
       <c r="Q68">
-        <f t="shared" si="5"/>
-        <v>0.45899999999999996</v>
+        <f t="shared" si="6"/>
+        <v>0.504</v>
       </c>
       <c r="R68">
         <f>R29+R26+R21+R5</f>
@@ -3864,63 +3726,63 @@
     </row>
     <row r="69" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B69" t="s">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="C69">
-        <f t="shared" ref="C69:M69" si="17">C30+C26+C21+C5</f>
+        <f t="shared" ref="C69:M69" si="18">C30+C26+C21+C5</f>
         <v>15</v>
       </c>
       <c r="D69">
+        <f t="shared" si="18"/>
+        <v>0.42000000000000004</v>
+      </c>
+      <c r="E69">
+        <f t="shared" si="18"/>
+        <v>-6</v>
+      </c>
+      <c r="F69">
+        <f t="shared" si="18"/>
+        <v>-20</v>
+      </c>
+      <c r="G69">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="H69">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="I69">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="J69">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="K69">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="L69">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="M69">
+        <f t="shared" si="18"/>
+        <v>1600</v>
+      </c>
+      <c r="N69">
         <f t="shared" si="17"/>
-        <v>0.4</v>
-      </c>
-      <c r="E69">
-        <f t="shared" si="17"/>
-        <v>-6</v>
-      </c>
-      <c r="F69">
-        <f t="shared" si="17"/>
-        <v>-20</v>
-      </c>
-      <c r="G69">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="H69">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="I69">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="J69">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="K69">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="L69">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="M69">
-        <f t="shared" si="17"/>
-        <v>1600</v>
-      </c>
-      <c r="N69">
-        <f t="shared" si="16"/>
-        <v>23.8</v>
+        <v>23.4</v>
       </c>
       <c r="P69">
         <f>P30+P26+P21+P5</f>
-        <v>17.8</v>
+        <v>20.8</v>
       </c>
       <c r="Q69">
-        <f t="shared" si="5"/>
-        <v>0.41700000000000004</v>
+        <f t="shared" si="6"/>
+        <v>0.46199999999999997</v>
       </c>
       <c r="R69">
         <f>R30+R26+R21+R5</f>
@@ -3933,63 +3795,63 @@
     </row>
     <row r="70" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B70" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C70">
-        <f t="shared" ref="C70:M70" si="18">C31+C32+C26+C21+C5</f>
+        <f t="shared" ref="C70:M70" si="19">C31+C32+C26+C21+C5</f>
         <v>18</v>
       </c>
       <c r="D70">
-        <f t="shared" si="18"/>
-        <v>0.30000000000000004</v>
+        <f t="shared" si="19"/>
+        <v>0.32000000000000006</v>
       </c>
       <c r="E70">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>-8</v>
       </c>
       <c r="F70">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>-9</v>
       </c>
       <c r="G70">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="H70">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="I70">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="J70">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="K70">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="L70">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="M70">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>1100</v>
       </c>
       <c r="N70">
-        <f t="shared" si="16"/>
-        <v>23.799999999999997</v>
+        <f t="shared" si="17"/>
+        <v>23.4</v>
       </c>
       <c r="P70">
         <f>P31+P32+P26+P21+P5</f>
-        <v>11.399999999999999</v>
+        <v>14.399999999999999</v>
       </c>
       <c r="Q70">
-        <f t="shared" si="5"/>
-        <v>0.32099999999999995</v>
+        <f t="shared" si="6"/>
+        <v>0.36599999999999999</v>
       </c>
       <c r="R70">
         <f>R31+R32+R26+R21+R5</f>
@@ -4002,63 +3864,63 @@
     </row>
     <row r="71" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B71" t="s">
-        <v>50</v>
+        <v>86</v>
       </c>
       <c r="C71">
-        <f t="shared" ref="C71:M71" si="19">C34+C33+C26+C21+C5</f>
+        <f t="shared" ref="C71:M71" si="20">C34+C33+C26+C21+C5</f>
         <v>17</v>
       </c>
       <c r="D71">
-        <f t="shared" si="19"/>
-        <v>0.35000000000000003</v>
+        <f t="shared" si="20"/>
+        <v>0.37</v>
       </c>
       <c r="E71">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>-11</v>
       </c>
       <c r="F71">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>-10</v>
       </c>
       <c r="G71">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="H71">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="I71">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="J71">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="K71">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="L71">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="M71">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>1400</v>
       </c>
       <c r="N71">
-        <f t="shared" si="16"/>
-        <v>24.8</v>
+        <f t="shared" si="17"/>
+        <v>24.4</v>
       </c>
       <c r="P71">
         <f>P34+P33+P26+P21+P5</f>
-        <v>13.2</v>
+        <v>16.2</v>
       </c>
       <c r="Q71">
-        <f t="shared" si="5"/>
-        <v>0.34799999999999998</v>
+        <f t="shared" si="6"/>
+        <v>0.39300000000000002</v>
       </c>
       <c r="R71">
         <f>R34+R33+R26+R21+R5</f>
@@ -4071,63 +3933,63 @@
     </row>
     <row r="72" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B72" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C72">
-        <f t="shared" ref="C72:M72" si="20">C36+C35+C26+C21+C5</f>
+        <f t="shared" ref="C72:M72" si="21">C36+C35+C26+C21+C5</f>
         <v>16</v>
       </c>
       <c r="D72">
-        <f t="shared" si="20"/>
-        <v>0.39</v>
+        <f t="shared" si="21"/>
+        <v>0.41000000000000003</v>
       </c>
       <c r="E72">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>-9</v>
       </c>
       <c r="F72">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>-14</v>
       </c>
       <c r="G72">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="H72">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="I72">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="J72">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="K72">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="L72">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="M72">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>1400</v>
       </c>
       <c r="N72">
-        <f t="shared" si="16"/>
-        <v>23.799999999999997</v>
+        <f t="shared" si="17"/>
+        <v>23.4</v>
       </c>
       <c r="P72">
         <f>P36+P35+P26+P21+P5</f>
-        <v>20.3</v>
+        <v>23.3</v>
       </c>
       <c r="Q72">
-        <f t="shared" si="5"/>
-        <v>0.45450000000000002</v>
+        <f t="shared" si="6"/>
+        <v>0.49949999999999994</v>
       </c>
       <c r="R72">
         <f>R36+R35+R26+R21+R5</f>
@@ -4140,63 +4002,63 @@
     </row>
     <row r="73" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B73" t="s">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="C73">
-        <f t="shared" ref="C73:M73" si="21">C38+C37+C26+C21+C5</f>
+        <f t="shared" ref="C73:M73" si="22">C38+C37+C26+C21+C5</f>
         <v>14</v>
       </c>
       <c r="D73">
-        <f t="shared" si="21"/>
-        <v>0.42500000000000004</v>
+        <f t="shared" si="22"/>
+        <v>0.44500000000000006</v>
       </c>
       <c r="E73">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>-12</v>
       </c>
       <c r="F73">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>-13</v>
       </c>
       <c r="G73">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="H73">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="I73">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="J73">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="K73">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="L73">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="M73">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>1300</v>
       </c>
       <c r="N73">
-        <f t="shared" si="16"/>
-        <v>22.900000000000002</v>
+        <f t="shared" si="17"/>
+        <v>22.5</v>
       </c>
       <c r="P73">
         <f>P38+P37+P26+P21+P5</f>
-        <v>18.8</v>
+        <v>21.8</v>
       </c>
       <c r="Q73">
-        <f t="shared" si="5"/>
-        <v>0.43199999999999994</v>
+        <f t="shared" si="6"/>
+        <v>0.47699999999999998</v>
       </c>
       <c r="R73">
         <f>R38+R37+R26+R21+R5</f>
@@ -4209,63 +4071,63 @@
     </row>
     <row r="74" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B74" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C74">
         <f>C41+C40+C39+C26+C21+C5</f>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D74">
-        <f t="shared" ref="D74:L74" si="22">D41+D40+D39+D26+D21+D5</f>
-        <v>0.56000000000000005</v>
+        <f t="shared" ref="D74:L74" si="23">D41+D40+D39+D26+D21+D5</f>
+        <v>0.58000000000000007</v>
       </c>
       <c r="E74">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>-6</v>
       </c>
       <c r="F74">
-        <f t="shared" si="22"/>
-        <v>-5</v>
+        <f t="shared" si="23"/>
+        <v>-18</v>
       </c>
       <c r="G74">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="H74">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>-0.05</v>
       </c>
       <c r="I74">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="J74">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="K74">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="L74">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="M74">
-        <f t="shared" ref="M74" si="23">M41+M40+M39+M26+M21+M5</f>
+        <f t="shared" ref="M74" si="24">M41+M40+M39+M26+M21+M5</f>
         <v>2100</v>
       </c>
       <c r="N74">
-        <f t="shared" si="16"/>
-        <v>16.850000000000001</v>
+        <f t="shared" si="17"/>
+        <v>22.25</v>
       </c>
       <c r="P74">
         <f>P41+P40+P39+P26+P21+P5</f>
-        <v>32.6</v>
+        <v>35.6</v>
       </c>
       <c r="Q74">
-        <f t="shared" si="5"/>
-        <v>0.63900000000000001</v>
+        <f t="shared" si="6"/>
+        <v>0.68400000000000005</v>
       </c>
       <c r="R74">
         <f>R41+R40+R39+R26+R21+R5</f>
@@ -4278,63 +4140,63 @@
     </row>
     <row r="75" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B75" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="C75">
         <f>C42+C26+C21+C5</f>
         <v>14</v>
       </c>
       <c r="D75">
-        <f t="shared" ref="D75:M75" si="24">D42+D26+D21+D5</f>
-        <v>0.35000000000000003</v>
+        <f t="shared" ref="D75:M75" si="25">D42+D26+D21+D5</f>
+        <v>0.37</v>
       </c>
       <c r="E75">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>-10</v>
       </c>
       <c r="F75">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>-13</v>
       </c>
       <c r="G75">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="H75">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="I75">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="J75">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="K75">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="L75">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="M75">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>1200</v>
       </c>
       <c r="N75">
-        <f t="shared" si="16"/>
-        <v>22.8</v>
+        <f t="shared" si="17"/>
+        <v>22.4</v>
       </c>
       <c r="P75">
         <f>P42+P26+P21+P5</f>
-        <v>14.3</v>
+        <v>17.3</v>
       </c>
       <c r="Q75">
-        <f t="shared" si="5"/>
-        <v>0.36449999999999999</v>
+        <f t="shared" si="6"/>
+        <v>0.40949999999999998</v>
       </c>
       <c r="R75">
         <f>R42+R26+R21+R5</f>
@@ -4347,63 +4209,63 @@
     </row>
     <row r="76" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B76" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C76">
         <f>C43+C26+C21+C5</f>
         <v>15</v>
       </c>
       <c r="D76">
-        <f t="shared" ref="D76:M76" si="25">D43+D26+D21+D5</f>
-        <v>0.36000000000000004</v>
+        <f t="shared" ref="D76:M76" si="26">D43+D26+D21+D5</f>
+        <v>0.38</v>
       </c>
       <c r="E76">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>-13</v>
       </c>
       <c r="F76">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>-8</v>
       </c>
       <c r="G76">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="H76">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="I76">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="J76">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="K76">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="L76">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="M76">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>1350</v>
       </c>
       <c r="N76">
-        <f t="shared" si="16"/>
-        <v>23</v>
+        <f t="shared" si="17"/>
+        <v>22.6</v>
       </c>
       <c r="P76">
         <f>P43+P26+P21+P5</f>
-        <v>14.8</v>
+        <v>17.8</v>
       </c>
       <c r="Q76">
-        <f t="shared" si="5"/>
-        <v>0.372</v>
+        <f t="shared" si="6"/>
+        <v>0.41700000000000004</v>
       </c>
       <c r="R76">
         <f>R43+R26+R21+R5</f>
@@ -4416,63 +4278,63 @@
     </row>
     <row r="77" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B77" t="s">
-        <v>68</v>
+        <v>89</v>
       </c>
       <c r="C77">
-        <f t="shared" ref="C77:M77" si="26">C44+C26+C21+C5</f>
+        <f t="shared" ref="C77:M77" si="27">C44+C26+C21+C5</f>
         <v>15</v>
       </c>
       <c r="D77">
-        <f t="shared" si="26"/>
-        <v>0.34</v>
+        <f t="shared" si="27"/>
+        <v>0.36000000000000004</v>
       </c>
       <c r="E77">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>-10</v>
       </c>
       <c r="F77">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>-8</v>
       </c>
       <c r="G77">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>0</v>
       </c>
       <c r="H77">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>0</v>
       </c>
       <c r="I77">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>0</v>
       </c>
       <c r="J77">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>0</v>
       </c>
       <c r="K77">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>0</v>
       </c>
       <c r="L77">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>0</v>
       </c>
       <c r="M77">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>600</v>
       </c>
       <c r="N77">
-        <f t="shared" si="16"/>
-        <v>21</v>
+        <f t="shared" si="17"/>
+        <v>20.599999999999998</v>
       </c>
       <c r="P77">
         <f>P44+P26+P21+P5</f>
-        <v>12.8</v>
+        <v>15.8</v>
       </c>
       <c r="Q77">
-        <f t="shared" si="5"/>
-        <v>0.34199999999999997</v>
+        <f t="shared" si="6"/>
+        <v>0.38700000000000001</v>
       </c>
       <c r="R77">
         <f>R44+R26+R21+R5</f>
@@ -4485,63 +4347,63 @@
     </row>
     <row r="78" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B78" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C78">
-        <f t="shared" ref="C78:M78" si="27">C46+C45+C26+C21+C5</f>
+        <f t="shared" ref="C78:M78" si="28">C46+C45+C26+C21+C5</f>
         <v>18</v>
       </c>
       <c r="D78">
-        <f t="shared" si="27"/>
-        <v>0.4</v>
+        <f t="shared" si="28"/>
+        <v>0.42000000000000004</v>
       </c>
       <c r="E78">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>-7</v>
       </c>
       <c r="F78">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>-15</v>
       </c>
       <c r="G78">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>0</v>
       </c>
       <c r="H78">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>0</v>
       </c>
       <c r="I78">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>0</v>
       </c>
       <c r="J78">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>0</v>
       </c>
       <c r="K78">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>0</v>
       </c>
       <c r="L78">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>0</v>
       </c>
       <c r="M78">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>1300</v>
       </c>
       <c r="N78">
-        <f t="shared" si="16"/>
-        <v>24.6</v>
+        <f t="shared" si="17"/>
+        <v>24.2</v>
       </c>
       <c r="P78">
         <f>P46+P45+P26+P21+P5</f>
-        <v>17.2</v>
+        <v>20.2</v>
       </c>
       <c r="Q78">
-        <f t="shared" si="5"/>
-        <v>0.40800000000000003</v>
+        <f t="shared" si="6"/>
+        <v>0.45299999999999996</v>
       </c>
       <c r="R78">
         <f>R46+R45+R26+R21+R5</f>
@@ -4554,63 +4416,63 @@
     </row>
     <row r="79" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B79" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C79">
-        <f t="shared" ref="C79:M79" si="28">C48+C47+C26+C21+C5</f>
+        <f t="shared" ref="C79:M79" si="29">C48+C47+C26+C21+C5</f>
         <v>16</v>
       </c>
       <c r="D79">
-        <f t="shared" si="28"/>
-        <v>0.31000000000000005</v>
+        <f t="shared" si="29"/>
+        <v>0.33000000000000007</v>
       </c>
       <c r="E79">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>-8</v>
       </c>
       <c r="F79">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>-13</v>
       </c>
       <c r="G79">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="H79">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="I79">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="J79">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="K79">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="L79">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="M79">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>1100</v>
       </c>
       <c r="N79">
-        <f t="shared" si="16"/>
-        <v>24</v>
+        <f t="shared" si="17"/>
+        <v>23.599999999999998</v>
       </c>
       <c r="P79">
         <f>P48+P47+P26+P21+P5</f>
-        <v>10.399999999999999</v>
+        <v>13.399999999999999</v>
       </c>
       <c r="Q79">
-        <f t="shared" si="5"/>
-        <v>0.30599999999999994</v>
+        <f t="shared" si="6"/>
+        <v>0.35099999999999998</v>
       </c>
       <c r="R79">
         <f>R48+R47+R26+R21+R5</f>
@@ -4623,63 +4485,63 @@
     </row>
     <row r="80" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B80" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C80">
-        <f t="shared" ref="C80:M80" si="29">C50+C49+C26+C21+C5</f>
+        <f t="shared" ref="C80:M80" si="30">C50+C49+C26+C21+C5</f>
         <v>17</v>
       </c>
       <c r="D80">
-        <f t="shared" si="29"/>
-        <v>0.39</v>
+        <f t="shared" si="30"/>
+        <v>0.41000000000000003</v>
       </c>
       <c r="E80">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>-11</v>
       </c>
       <c r="F80">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>-11</v>
       </c>
       <c r="G80">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="H80">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="I80">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="J80">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="K80">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="L80">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="M80">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>1500</v>
       </c>
       <c r="N80">
-        <f t="shared" si="16"/>
-        <v>24.6</v>
+        <f t="shared" si="17"/>
+        <v>24.200000000000003</v>
       </c>
       <c r="P80">
         <f>P50+P49+P26+P21+P5</f>
-        <v>17.399999999999999</v>
+        <v>20.399999999999999</v>
       </c>
       <c r="Q80">
-        <f t="shared" si="5"/>
-        <v>0.41099999999999992</v>
+        <f t="shared" si="6"/>
+        <v>0.45599999999999996</v>
       </c>
       <c r="R80">
         <f>R50+R49+R26+R21+R5</f>
@@ -4692,63 +4554,63 @@
     </row>
     <row r="81" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B81" t="s">
-        <v>106</v>
+        <v>74</v>
       </c>
       <c r="C81">
-        <f t="shared" ref="C81:M81" si="30">C52+C51+C26+C21+C5</f>
+        <f t="shared" ref="C81:M81" si="31">C52+C51+C26+C21+C5</f>
         <v>18</v>
       </c>
       <c r="D81">
         <f>D52+D51+D26+D21+D5</f>
-        <v>0.33</v>
+        <v>0.35000000000000003</v>
       </c>
       <c r="E81">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>-9</v>
       </c>
       <c r="F81">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>-10</v>
       </c>
       <c r="G81">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="H81">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="I81">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="J81">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="K81">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="L81">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="M81">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>1400</v>
       </c>
       <c r="N81">
-        <f t="shared" si="16"/>
-        <v>24.599999999999998</v>
+        <f t="shared" si="17"/>
+        <v>24.2</v>
       </c>
       <c r="P81">
         <f>P52+P51+P26+P21+P5</f>
-        <v>12.6</v>
+        <v>15.6</v>
       </c>
       <c r="Q81">
-        <f t="shared" si="5"/>
-        <v>0.33899999999999997</v>
+        <f t="shared" si="6"/>
+        <v>0.38400000000000001</v>
       </c>
       <c r="R81">
         <f>R52+R51+R26+R21+R5</f>
@@ -4761,63 +4623,63 @@
     </row>
     <row r="82" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B82" t="s">
-        <v>113</v>
+        <v>76</v>
       </c>
       <c r="C82">
-        <f t="shared" ref="C82:M82" si="31">C54+C53+C26+C21+C5</f>
+        <f t="shared" ref="C82:M82" si="32">C54+C53+C26+C21+C5</f>
         <v>16</v>
       </c>
       <c r="D82">
-        <f t="shared" si="31"/>
-        <v>0.34</v>
+        <f t="shared" si="32"/>
+        <v>0.36</v>
       </c>
       <c r="E82">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>-10</v>
       </c>
       <c r="F82">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>-12</v>
       </c>
       <c r="G82">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>0</v>
       </c>
       <c r="H82">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>0</v>
       </c>
       <c r="I82">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>0</v>
       </c>
       <c r="J82">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>0</v>
       </c>
       <c r="K82">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>0</v>
       </c>
       <c r="L82">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>0</v>
       </c>
       <c r="M82">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>1500</v>
       </c>
       <c r="N82">
-        <f t="shared" si="16"/>
-        <v>24.4</v>
+        <f t="shared" si="17"/>
+        <v>24</v>
       </c>
       <c r="P82">
         <f>P54+P53+P26+P21+P5</f>
-        <v>12.8</v>
+        <v>15.8</v>
       </c>
       <c r="Q82">
-        <f t="shared" si="5"/>
-        <v>0.34199999999999997</v>
+        <f t="shared" si="6"/>
+        <v>0.38700000000000001</v>
       </c>
       <c r="R82">
         <f>R54+R53+R26+R21+R5</f>
@@ -4830,6 +4692,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>